<commit_message>
#6 DB-9 Connector part no Update in Power PCB
</commit_message>
<xml_diff>
--- a/Design Files/Power-PCB/BOM/Power-PCB.xlsx
+++ b/Design Files/Power-PCB/BOM/Power-PCB.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\eamonelkhedrawi-boarddesign\Design Files\Power-PCB\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="56">
   <si>
     <t>#</t>
   </si>
@@ -119,12 +124,6 @@
     <t>CONN D-SUB RCPT 9POS R/A SLDR</t>
   </si>
   <si>
-    <t>A-DF 09 A/KG-T2S</t>
-  </si>
-  <si>
-    <t>Assmann</t>
-  </si>
-  <si>
     <t>Relays</t>
   </si>
   <si>
@@ -189,19 +188,25 @@
   </si>
   <si>
     <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>LX09-VGA09B-048</t>
+  </si>
+  <si>
+    <t>Lian Xin Technology</t>
+  </si>
+  <si>
+    <t>CRCW0603220RFKEA</t>
+  </si>
+  <si>
+    <t>Vishay</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -213,14 +218,14 @@
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -228,168 +233,24 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -408,194 +269,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -686,251 +361,9 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -973,67 +406,23 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1291,28 +680,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
-    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
-    <col min="9" max="9" width="17.8571428571429" customWidth="1"/>
-    <col min="10" max="10" width="16.7142857142857" customWidth="1"/>
-    <col min="11" max="11" width="29.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1325,7 +715,7 @@
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
     </row>
-    <row r="2" ht="15.75" spans="1:11">
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1358,7 +748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="15.75" spans="1:11">
+    <row r="3" spans="1:11">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
         <f>ROW(B3)-ROW($B$2)</f>
@@ -1390,7 +780,7 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" ht="60.75" spans="1:11">
+    <row r="4" spans="1:11" ht="60">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
         <f t="shared" ref="B4:B10" si="0">ROW(B4)-ROW($B$2)</f>
@@ -1422,7 +812,7 @@
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" ht="60.75" spans="1:11">
+    <row r="5" spans="1:11" ht="60">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
         <f t="shared" si="0"/>
@@ -1454,7 +844,7 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" ht="15.75" spans="1:11">
+    <row r="6" spans="1:11">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
         <f t="shared" si="0"/>
@@ -1473,10 +863,10 @@
         <v>20</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="I6" s="13" t="s">
         <v>23</v>
@@ -1486,29 +876,29 @@
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="36.75" spans="1:11">
+    <row r="7" spans="1:11" ht="36">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>32</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>34</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>23</v>
@@ -1518,29 +908,29 @@
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" ht="15.75" spans="1:11">
+    <row r="8" spans="1:11">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="F8" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="G8" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="H8" s="12" t="s">
         <v>40</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>42</v>
       </c>
       <c r="I8" s="13" t="s">
         <v>23</v>
@@ -1550,57 +940,61 @@
       </c>
       <c r="K8" s="12"/>
     </row>
-    <row r="9" ht="15.75" spans="1:11">
+    <row r="9" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="G9" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="10" t="s">
-        <v>47</v>
       </c>
       <c r="J9" s="9">
         <v>6</v>
       </c>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" ht="15.75" spans="1:11">
+    <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="F10" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="G10" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="H10" s="12" t="s">
         <v>51</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>53</v>
       </c>
       <c r="I10" s="13" t="s">
         <v>23</v>
@@ -1616,6 +1010,5 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>